<commit_message>
Web app: password reset, dropdown + country fixes, CSV import, report polish
</commit_message>
<xml_diff>
--- a/docs/pilot/EnergyLens_Pilot_Data_Intake.xlsx
+++ b/docs/pilot/EnergyLens_Pilot_Data_Intake.xlsx
@@ -8,9 +8,11 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start here" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 About you" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Buildings" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Data availability" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Building &amp; energy" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 About you" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Buildings" sheetId="4" state="hidden" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Data availability" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Systems &amp; sources" sheetId="6" state="hidden" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,8 +67,45 @@
       <color rgb="001F6B53"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00606060"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -83,8 +122,18 @@
         <fgColor rgb="00DCEAE3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8EEF7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -106,11 +155,69 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -139,6 +246,36 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -550,23 +687,15 @@
     <row r="9">
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>•  Tab 1 — About you &amp; your portfolio (and a few quick questions).</t>
+          <t>•  Just fill the “Building &amp; energy” tab — only the yellow cells. About 5 minutes.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>•  Tab 2 — List your buildings (one row each).</t>
-        </is>
-      </c>
+      <c r="B10" s="4" t="n"/>
     </row>
     <row r="11">
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>•  Tab 3 — Tick which data you can share (Yes / Partial / No). This is the detailed part; skip rows that don't apply.</t>
-        </is>
-      </c>
+      <c r="B11" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
@@ -609,6 +738,372 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>EnergyLens — Building &amp; energy (quick form)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="21" t="inlineStr">
+        <is>
+          <t>Fill the yellow cells. Where you see a dropdown arrow, just pick. Numbers only — the unit is already shown. About 5 minutes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="22" t="inlineStr">
+        <is>
+          <t>About you</t>
+        </is>
+      </c>
+      <c r="B4" s="23" t="n"/>
+      <c r="C4" s="23" t="n"/>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="24" t="inlineStr">
+        <is>
+          <t>Your name</t>
+        </is>
+      </c>
+      <c r="B5" s="25" t="n"/>
+      <c r="C5" s="26" t="inlineStr"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>Company / organisation</t>
+        </is>
+      </c>
+      <c r="B6" s="25" t="n"/>
+      <c r="C6" s="26" t="inlineStr"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="24" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="B7" s="25" t="n"/>
+      <c r="C7" s="26" t="inlineStr"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="22" t="inlineStr">
+        <is>
+          <t>Your building</t>
+        </is>
+      </c>
+      <c r="B9" s="23" t="n"/>
+      <c r="C9" s="23" t="n"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>Building name</t>
+        </is>
+      </c>
+      <c r="B10" s="25" t="n"/>
+      <c r="C10" s="26" t="inlineStr"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="24" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="B11" s="25" t="n"/>
+      <c r="C11" s="26" t="inlineStr"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="24" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="B12" s="25" t="n"/>
+      <c r="C12" s="26" t="inlineStr"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="24" t="inlineStr">
+        <is>
+          <t>Use type</t>
+        </is>
+      </c>
+      <c r="B13" s="25" t="n"/>
+      <c r="C13" s="26" t="inlineStr"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="24" t="inlineStr">
+        <is>
+          <t>Gross floor area (m²)</t>
+        </is>
+      </c>
+      <c r="B14" s="25" t="n"/>
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="24" t="inlineStr">
+        <is>
+          <t>Year built</t>
+        </is>
+      </c>
+      <c r="B15" s="25" t="n"/>
+      <c r="C15" s="26" t="inlineStr">
+        <is>
+          <t>approx. is fine</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="24" t="inlineStr">
+        <is>
+          <t>Main heating source</t>
+        </is>
+      </c>
+      <c r="B16" s="25" t="n"/>
+      <c r="C16" s="26" t="inlineStr">
+        <is>
+          <t>heating AND electricity both matter for correct numbers</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="22" t="inlineStr">
+        <is>
+          <t>Energy use (last 12 months)</t>
+        </is>
+      </c>
+      <c r="B18" s="23" t="n"/>
+      <c r="C18" s="23" t="n"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="24" t="inlineStr">
+        <is>
+          <t>Electricity total (kWh/year)</t>
+        </is>
+      </c>
+      <c r="B19" s="25" t="n"/>
+      <c r="C19" s="26" t="inlineStr">
+        <is>
+          <t>or just send 12 monthly bills and I will read them</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="24" t="inlineStr">
+        <is>
+          <t>Heating total (kWh/year)</t>
+        </is>
+      </c>
+      <c r="B20" s="25" t="n"/>
+      <c r="C20" s="26" t="inlineStr">
+        <is>
+          <t>gas / district heat; bills are fine too</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="22" t="inlineStr">
+        <is>
+          <t>Systems present (pick Yes/No, add the number if yes)</t>
+        </is>
+      </c>
+      <c r="B22" s="23" t="n"/>
+      <c r="C22" s="23" t="n"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="24" t="inlineStr">
+        <is>
+          <t>Solar PV?</t>
+        </is>
+      </c>
+      <c r="B23" s="25" t="n"/>
+      <c r="C23" s="26" t="inlineStr"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ PV size (kWp)</t>
+        </is>
+      </c>
+      <c r="B24" s="25" t="n"/>
+      <c r="C24" s="26" t="inlineStr">
+        <is>
+          <t>only if PV = Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="24" t="inlineStr">
+        <is>
+          <t>Battery?</t>
+        </is>
+      </c>
+      <c r="B25" s="25" t="n"/>
+      <c r="C25" s="26" t="inlineStr"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ Battery size (kWh)</t>
+        </is>
+      </c>
+      <c r="B26" s="25" t="n"/>
+      <c r="C26" s="26" t="inlineStr">
+        <is>
+          <t>only if Battery = Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="24" t="inlineStr">
+        <is>
+          <t>Heat pump?</t>
+        </is>
+      </c>
+      <c r="B27" s="25" t="n"/>
+      <c r="C27" s="26" t="inlineStr"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ Heat pump output (kW)</t>
+        </is>
+      </c>
+      <c r="B28" s="25" t="n"/>
+      <c r="C28" s="26" t="inlineStr">
+        <is>
+          <t>only if Heat pump = Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ Heat pump COP</t>
+        </is>
+      </c>
+      <c r="B29" s="25" t="n"/>
+      <c r="C29" s="26" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="24" t="inlineStr">
+        <is>
+          <t>EV charging?</t>
+        </is>
+      </c>
+      <c r="B30" s="25" t="n"/>
+      <c r="C30" s="26" t="inlineStr"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="24" t="inlineStr">
+        <is>
+          <t>Sub-meters per floor or system?</t>
+        </is>
+      </c>
+      <c r="B31" s="25" t="n"/>
+      <c r="C31" s="26" t="inlineStr"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="24" t="inlineStr">
+        <is>
+          <t>BMS / building automation</t>
+        </is>
+      </c>
+      <c r="B32" s="25" t="n"/>
+      <c r="C32" s="26" t="inlineStr"/>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="22" t="inlineStr">
+        <is>
+          <t>Sharing</t>
+        </is>
+      </c>
+      <c r="B34" s="23" t="n"/>
+      <c r="C34" s="23" t="n"/>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="24" t="inlineStr">
+        <is>
+          <t>How will you share data?</t>
+        </is>
+      </c>
+      <c r="B35" s="25" t="n"/>
+      <c r="C35" s="26" t="inlineStr"/>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="24" t="inlineStr">
+        <is>
+          <t>Anything else / questions</t>
+        </is>
+      </c>
+      <c r="B36" s="25" t="n"/>
+      <c r="C36" s="26" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <dataValidations count="10">
+    <dataValidation sqref="B12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"DE,AT,NL,TR,Other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Office,Retail,Hotel,Healthcare,Education,Logistics/Warehouse,Residential (MFH),Mixed-use,Other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Natural gas,District heating,Heat pump,Oil,Biomass or pellets,Electric direct,Mixed,None"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"None,Siemens Desigo,Schneider EcoStruxure,Honeywell,Johnson Controls Metasys,Bosch,Kieback&amp;Peter,Priva,Other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Utility bills (PDF or scan),Excel or CSV export,BMS or BAS export,Smart-meter portal,Manufacturer cloud or API,Other"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -786,7 +1281,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1017,7 +1512,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1054,8 +1549,8 @@
           <t>A. Building &amp; occupancy</t>
         </is>
       </c>
-      <c r="B2" s="8" t="n"/>
-      <c r="C2" s="8" t="n"/>
+      <c r="B2" s="13" t="n"/>
+      <c r="C2" s="14" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
@@ -1090,8 +1585,8 @@
           <t>B. Electricity</t>
         </is>
       </c>
-      <c r="B6" s="8" t="n"/>
-      <c r="C6" s="8" t="n"/>
+      <c r="B6" s="13" t="n"/>
+      <c r="C6" s="14" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
@@ -1135,8 +1630,8 @@
           <t>C. Heating</t>
         </is>
       </c>
-      <c r="B11" s="8" t="n"/>
-      <c r="C11" s="8" t="n"/>
+      <c r="B11" s="13" t="n"/>
+      <c r="C11" s="14" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
@@ -1171,8 +1666,8 @@
           <t>D. Heat pump</t>
         </is>
       </c>
-      <c r="B15" s="8" t="n"/>
-      <c r="C15" s="8" t="n"/>
+      <c r="B15" s="13" t="n"/>
+      <c r="C15" s="14" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
@@ -1216,8 +1711,8 @@
           <t>E. HVAC equipment</t>
         </is>
       </c>
-      <c r="B20" s="8" t="n"/>
-      <c r="C20" s="8" t="n"/>
+      <c r="B20" s="13" t="n"/>
+      <c r="C20" s="14" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
@@ -1243,8 +1738,8 @@
           <t>F. Sub-metering</t>
         </is>
       </c>
-      <c r="B23" s="8" t="n"/>
-      <c r="C23" s="8" t="n"/>
+      <c r="B23" s="13" t="n"/>
+      <c r="C23" s="14" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
@@ -1261,8 +1756,8 @@
           <t>G. BMS / BAS &amp; IoT</t>
         </is>
       </c>
-      <c r="B25" s="8" t="n"/>
-      <c r="C25" s="8" t="n"/>
+      <c r="B25" s="13" t="n"/>
+      <c r="C25" s="14" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
@@ -1297,8 +1792,8 @@
           <t>H. Solar PV</t>
         </is>
       </c>
-      <c r="B29" s="8" t="n"/>
-      <c r="C29" s="8" t="n"/>
+      <c r="B29" s="13" t="n"/>
+      <c r="C29" s="14" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="12" t="inlineStr">
@@ -1333,8 +1828,8 @@
           <t>I. Battery storage (BESS)</t>
         </is>
       </c>
-      <c r="B33" s="8" t="n"/>
-      <c r="C33" s="8" t="n"/>
+      <c r="B33" s="13" t="n"/>
+      <c r="C33" s="14" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="12" t="inlineStr">
@@ -1360,8 +1855,8 @@
           <t>J. EV charging</t>
         </is>
       </c>
-      <c r="B36" s="8" t="n"/>
-      <c r="C36" s="8" t="n"/>
+      <c r="B36" s="13" t="n"/>
+      <c r="C36" s="14" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="12" t="inlineStr">
@@ -1378,8 +1873,8 @@
           <t>K. Refrigerant / F-Gas</t>
         </is>
       </c>
-      <c r="B38" s="8" t="n"/>
-      <c r="C38" s="8" t="n"/>
+      <c r="B38" s="13" t="n"/>
+      <c r="C38" s="14" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="12" t="inlineStr">
@@ -1396,8 +1891,8 @@
           <t>L. Envelope &amp; EPC</t>
         </is>
       </c>
-      <c r="B40" s="8" t="n"/>
-      <c r="C40" s="8" t="n"/>
+      <c r="B40" s="13" t="n"/>
+      <c r="C40" s="14" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="12" t="inlineStr">
@@ -1423,8 +1918,8 @@
           <t>M. Compliance &amp; ESG context</t>
         </is>
       </c>
-      <c r="B43" s="8" t="n"/>
-      <c r="C43" s="8" t="n"/>
+      <c r="B43" s="13" t="n"/>
+      <c r="C43" s="14" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="12" t="inlineStr">
@@ -1459,8 +1954,8 @@
           <t>N. Residential (multi-family, if applicable)</t>
         </is>
       </c>
-      <c r="B47" s="8" t="n"/>
-      <c r="C47" s="8" t="n"/>
+      <c r="B47" s="13" t="n"/>
+      <c r="C47" s="14" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="12" t="inlineStr">
@@ -1502,8 +1997,8 @@
   <mergeCells count="14">
     <mergeCell ref="A25:C25"/>
     <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A36:C36"/>
     <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A36:C36"/>
     <mergeCell ref="A47:C47"/>
     <mergeCell ref="A23:C23"/>
     <mergeCell ref="A43:C43"/>
@@ -1522,4 +2017,266 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>EnergyLens — Systems &amp; data sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>Optional but very helpful. Just pick from the dropdowns (about 2 minutes). It tells me exactly how to take your data with zero effort on your side.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>Your answer (pick from list)</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>Notes / details (optional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>How will you share data?</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="n"/>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>Pick the easiest one for you</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Metering setup</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="n"/>
+      <c r="C6" s="19" t="inlineStr"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>Granularity you can provide</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="n"/>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>Monthly is already enough to start</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Electricity data source</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="n"/>
+      <c r="C8" s="19" t="inlineStr"/>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>Heating source</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="n"/>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>I need heating AND electricity for correct numbers</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>Heat pump cloud / API (if any)</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="n"/>
+      <c r="C10" s="19" t="inlineStr"/>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>BMS / BAS system (brand)</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="n"/>
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>If you have building automation</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>Field protocols available</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="n"/>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>Only if BMS or live sensors exist</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>Solar PV monitoring (if any)</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="n"/>
+      <c r="C13" s="19" t="inlineStr"/>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>Heat-cost allocation provider (residential)</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="n"/>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>Techem / ista etc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>Existing energy / ESG software</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="n"/>
+      <c r="C15" s="19" t="inlineStr"/>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>Read-only export or API access possible?</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="n"/>
+      <c r="C16" s="19" t="inlineStr"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>Preferred transfer method</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="n"/>
+      <c r="C17" s="19" t="inlineStr"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>Utility / DSO / provider names</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="n"/>
+      <c r="C18" s="19" t="inlineStr">
+        <is>
+          <t>Free text</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>Anything else about your systems</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="n"/>
+      <c r="C19" s="19" t="inlineStr">
+        <is>
+          <t>Free text</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <dataValidations count="13">
+    <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Utility bills (PDF or scan),Excel or CSV export,BMS or BAS export file,Smart-meter portal export,Manufacturer cloud or API,Manual entry in this file,Other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Utility bills only,Smart meter(s),Sub-meters per system,Full BMS or BAS,Mix of these,Not sure"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Monthly,Daily,Hourly,15-minute,Mixed,Not sure"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Utility bill,DSO or smart-meter portal,Sub-meter or BMS,MSCONS/EDIFACT file,Other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Natural gas,District heating,Heat pump,Oil,Biomass or pellets,Electric direct,Mixed,None"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Viessmann,Vaillant,Bosch or Buderus,Daikin,Mitsubishi,Stiebel Eltron,NIBE,None,Other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Siemens Desigo,Schneider EcoStruxure,Honeywell,Johnson Controls Metasys,Bosch,Kieback&amp;Peter,Priva,Trend,Distech,Sauter,WAGO,None,Other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"BACnet/IP,Modbus TCP,Modbus RTU,MQTT,OPC-UA,REST/HTTP API,KNX,M-Bus,LoRaWAN,None or unknown,Other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"SolarEdge,SMA,Fronius,Huawei,Kostal,Other,None"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Techem,ista,Brunata-Minol,Minol,KALO,None,Other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"None,Excel only,EnergyCAP,Predium,Deepki,aedifion,Other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No,Maybe"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Email attachment,Shared link you provide,Upload link I send you,Other"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>